<commit_message>
Visão geral em cards (estilo Pós-Corte), escopo das 10 equipes/12 cidades e aba de tempos
- Visão geral: Percorrido/Exec/Exoc/Com resultados, tipos de resultado,
  bases, resultado por equipe (com "+" que abre os serviços) e por data;
  volta ao visual de cards do painel de Pós-Corte (claro/escuro)
- Escopo fixo: RIORECIN-004/007/013/024/034 e RIOVENIN-001 a 005, nas 12
  cidades do interior; o resto não entra nos números (auditoria mostra)
- Aba Tempos das equipes: deslocamento, serviço, pausas/apoio e
  ociosidade por equipe (média por dia ou total), só dias completos por padrão
- Removidas as matrizes e colunas de desfecho; Novos alvos e Auditoria mantidas
- Dados guardados por versão antiga são descartados e relidos da pasta
- Testes (83), README e docs atualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KJXQpbPz16uD2PcQ4EsKpx
</commit_message>
<xml_diff>
--- a/exemplos/exemplo-atividades.xlsx
+++ b/exemplos/exemplo-atividades.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RIORECIN-001</t>
+          <t>RIORECIN-004</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -576,7 +576,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RIORECIN-001</t>
+          <t>RIORECIN-004</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -794,7 +794,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>RIORECIN-001</t>
+          <t>RIORECIN-004</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -865,7 +865,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1078,16 +1078,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RIOCORTE-001</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1000009/2026-1</t>
+          <t>1000010/2026-1</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D10" t="n">
         <v>100000008</v>
@@ -1098,11 +1098,11 @@
         </is>
       </c>
       <c r="F10" s="1" t="n">
-        <v>46086</v>
+        <v>46087</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Finalizada</t>
+          <t>Encerrada com Ocorrência</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1127,7 +1127,12 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Corte e Religação Cavalete</t>
+          <t>Verificação Cadastral</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>RETORNAR DEPOIS</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1137,23 +1142,28 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Sem observação de abertura</t>
+          <t>PROJETO INCREMENTO: VERIFICAR O TIPO E A QUANTIDADE DE ECONOMIAS EXISTENTES. CASO HAJA MAIS DE UMA, OFERECER DESMEMBRAMENTO/VENDA.</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>01. ECON</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>1000010/2026-1</t>
+          <t>1000011/2026-1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D11" t="n">
         <v>100000008</v>
@@ -1168,7 +1178,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Encerrada com Ocorrência</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1194,11 +1204,6 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>Verificação Cadastral</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>RETORNAR DEPOIS</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1220,19 +1225,19 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1000011/2026-1</t>
+          <t>1000012/2026-1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" t="n">
-        <v>100000008</v>
+        <v>100000010</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1254,7 +1259,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>MIRACEMA</t>
+          <t>CORDEIRO</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1264,7 +1269,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>MIRACEMA - SETOR 002</t>
+          <t>CORDEIRO - SETOR 001</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1279,7 +1284,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>PROJETO INCREMENTO: VERIFICAR O TIPO E A QUANTIDADE DE ECONOMIAS EXISTENTES. CASO HAJA MAIS DE UMA, OFERECER DESMEMBRAMENTO/VENDA.</t>
+          <t>Sem observação de abertura</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1291,19 +1296,19 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1000012/2026-1</t>
+          <t>1000013/2026-1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" t="n">
-        <v>100000010</v>
+        <v>12345</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1350,7 +1355,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Sem observação de abertura</t>
+          <t>PROJETO INCREMENTO: VERIFICAR O TIPO E A QUANTIDADE DE ECONOMIAS EXISTENTES. CASO HAJA MAIS DE UMA, OFERECER DESMEMBRAMENTO/VENDA.</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1362,19 +1367,19 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIORECIN-007</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1000013/2026-1</t>
+          <t>1000014/2026-1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D14" t="n">
-        <v>12345</v>
+        <v>100000011</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1421,7 +1426,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>PROJETO INCREMENTO: VERIFICAR O TIPO E A QUANTIDADE DE ECONOMIAS EXISTENTES. CASO HAJA MAIS DE UMA, OFERECER DESMEMBRAMENTO/VENDA.</t>
+          <t>LNA - VARREDURA - FAVOR IDENTIFICAR O CLIENTE E FAZER VENDA DE LIGACAO NOVA.</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1433,19 +1438,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>RIORECIN-002</t>
+          <t>RIOVENIN-001</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1000014/2026-1</t>
+          <t>1000015/2026-1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" t="n">
-        <v>100000011</v>
+        <v>100000009</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1467,7 +1472,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>CORDEIRO</t>
+          <t>MIRACEMA</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1477,7 +1482,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>CORDEIRO - SETOR 001</t>
+          <t>MIRACEMA - SETOR 002</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1492,7 +1497,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>LNA - VARREDURA - FAVOR IDENTIFICAR O CLIENTE E FAZER VENDA DE LIGACAO NOVA.</t>
+          <t>PROJETO TITULARIDADE: FAVOR IDENTIFICAR O CLIENTE E FAZER TROCA DE TITULARIDADE.</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1504,19 +1509,19 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RIOVENIN-001</t>
+          <t>RIORECIN-004</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1000015/2026-1</t>
+          <t>1000016/2026-1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D16" t="n">
-        <v>100000009</v>
+        <v>100000012</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1524,7 +1529,7 @@
         </is>
       </c>
       <c r="F16" s="1" t="n">
-        <v>46087</v>
+        <v>46083</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1548,7 +1553,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>MIRACEMA - SETOR 002</t>
+          <t>MIRACEMA - SETOR 001</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1563,7 +1568,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>PROJETO TITULARIDADE: FAVOR IDENTIFICAR O CLIENTE E FAZER TROCA DE TITULARIDADE.</t>
+          <t>PROJETO INCREMENTO: VERIFICAR O TIPO E A QUANTIDADE DE ECONOMIAS EXISTENTES. CASO HAJA MAIS DE UMA, OFERECER DESMEMBRAMENTO/VENDA.</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1575,16 +1580,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RIORECIN-001</t>
+          <t>RIORECIN-004</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1000016/2026-1</t>
+          <t>1000017/2026-1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D17" t="n">
         <v>100000012</v>
@@ -1595,7 +1600,7 @@
         </is>
       </c>
       <c r="F17" s="1" t="n">
-        <v>46083</v>
+        <v>46093</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1638,77 +1643,6 @@
         </is>
       </c>
       <c r="P17" t="inlineStr">
-        <is>
-          <t>01. ECON</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>RIORECIN-001</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>1000017/2026-1</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>17</v>
-      </c>
-      <c r="D18" t="n">
-        <v>100000012</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>202012-VISTORIA DE RECADASTRO</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="n">
-        <v>46093</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Finalizada</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>RUA TESTE, 1</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>MIRACEMA</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>CENTRO</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>MIRACEMA - SETOR 001</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Verificação Cadastral</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>R-RESIDENCIAL</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>PROJETO INCREMENTO: VERIFICAR O TIPO E A QUANTIDADE DE ECONOMIAS EXISTENTES. CASO HAJA MAIS DE UMA, OFERECER DESMEMBRAMENTO/VENDA.</t>
-        </is>
-      </c>
-      <c r="P18" t="inlineStr">
         <is>
           <t>01. ECON</t>
         </is>

</xml_diff>